<commit_message>
เพิ่ม ESP32-S3 WROOM 1U / ร้าน Lantern IoT Maker กับ MASSMORE จาก Shopee
- เพิ่ม ESP32-S3 WROOM 1U
- Link Shopee ของร้าน Lantern IoT Maker
- Link Shopee ของร้าน MASSMORE
</commit_message>
<xml_diff>
--- a/List อุปกรณ์.xlsx
+++ b/List อุปกรณ์.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Classroom\มหาลัย\ปี 3\Project\AI-Powered-3D-Fall-Detection-System-using-WiFi-Sensing\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{25AB0289-B579-4FE6-8B34-C6710C8CB66F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D9573740-C013-4DB6-8E57-0C79399149FA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13176" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="66" uniqueCount="51">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="129" uniqueCount="58">
   <si>
     <t>List</t>
   </si>
@@ -173,13 +173,34 @@
   </si>
   <si>
     <t>MASSMORE - Shopee</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ESP32-S3-WROOM </t>
+  </si>
+  <si>
+    <t>185 - 239</t>
+  </si>
+  <si>
+    <t>โมดูลชิพ WROOM32 แท้จาก Espressif</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ESP32 WROOM-32E WROOM-32U </t>
+  </si>
+  <si>
+    <t>WiFi BLE PCB Antenna IPEX connector</t>
+  </si>
+  <si>
+    <t>ตัวเลือกสินค้า มีแบบเสาใน PCB Antenna</t>
+  </si>
+  <si>
+    <t>และเสานอก IPEX connector</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="11" x14ac:knownFonts="1">
+  <fonts count="12" x14ac:knownFonts="1">
     <font>
       <sz val="10"/>
       <color rgb="FF000000"/>
@@ -251,6 +272,14 @@
       <color rgb="FF000000"/>
       <name val="Times New Roman"/>
       <family val="1"/>
+    </font>
+    <font>
+      <u/>
+      <sz val="10"/>
+      <color theme="10"/>
+      <name val="Arial"/>
+      <family val="2"/>
+      <scheme val="minor"/>
     </font>
   </fonts>
   <fills count="8">
@@ -386,7 +415,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="26">
+  <cellXfs count="27">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
@@ -412,17 +441,10 @@
     <xf numFmtId="0" fontId="1" fillId="6" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="6" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="6" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="1" fillId="6" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="8" fillId="7" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="8" fillId="7" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="8" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
@@ -444,7 +466,19 @@
     <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="1"/>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="1" applyFont="1"/>
+    <xf numFmtId="0" fontId="8" fillId="6" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="6" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
@@ -681,50 +715,50 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:42" ht="33.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="13" t="s">
+      <c r="A1" s="23" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="14"/>
-      <c r="C1" s="14"/>
-      <c r="D1" s="14"/>
-      <c r="E1" s="14"/>
-      <c r="F1" s="14"/>
-      <c r="G1" s="17"/>
-      <c r="H1" s="18"/>
-      <c r="I1" s="19"/>
-      <c r="J1" s="20"/>
-      <c r="K1" s="20"/>
-      <c r="L1" s="20"/>
-      <c r="M1" s="20"/>
-      <c r="N1" s="20"/>
-      <c r="O1" s="20"/>
-      <c r="P1" s="21"/>
-      <c r="Q1" s="22"/>
-      <c r="R1" s="22"/>
-      <c r="S1" s="22"/>
-      <c r="T1" s="22"/>
-      <c r="U1" s="22"/>
-      <c r="V1" s="22"/>
-      <c r="W1" s="22"/>
-      <c r="X1" s="22"/>
-      <c r="Y1" s="22"/>
-      <c r="Z1" s="22"/>
-      <c r="AA1" s="22"/>
-      <c r="AB1" s="22"/>
-      <c r="AC1" s="22"/>
-      <c r="AD1" s="22"/>
-      <c r="AE1" s="22"/>
-      <c r="AF1" s="22"/>
-      <c r="AG1" s="22"/>
-      <c r="AH1" s="22"/>
-      <c r="AI1" s="22"/>
-      <c r="AJ1" s="22"/>
-      <c r="AK1" s="22"/>
-      <c r="AL1" s="22"/>
-      <c r="AM1" s="22"/>
-      <c r="AN1" s="22"/>
-      <c r="AO1" s="22"/>
-      <c r="AP1" s="22"/>
+      <c r="B1" s="24"/>
+      <c r="C1" s="24"/>
+      <c r="D1" s="24"/>
+      <c r="E1" s="24"/>
+      <c r="F1" s="24"/>
+      <c r="G1" s="14"/>
+      <c r="H1" s="15"/>
+      <c r="I1" s="16"/>
+      <c r="J1" s="17"/>
+      <c r="K1" s="17"/>
+      <c r="L1" s="17"/>
+      <c r="M1" s="17"/>
+      <c r="N1" s="17"/>
+      <c r="O1" s="17"/>
+      <c r="P1" s="18"/>
+      <c r="Q1" s="19"/>
+      <c r="R1" s="19"/>
+      <c r="S1" s="19"/>
+      <c r="T1" s="19"/>
+      <c r="U1" s="19"/>
+      <c r="V1" s="19"/>
+      <c r="W1" s="19"/>
+      <c r="X1" s="19"/>
+      <c r="Y1" s="19"/>
+      <c r="Z1" s="19"/>
+      <c r="AA1" s="19"/>
+      <c r="AB1" s="19"/>
+      <c r="AC1" s="19"/>
+      <c r="AD1" s="19"/>
+      <c r="AE1" s="19"/>
+      <c r="AF1" s="19"/>
+      <c r="AG1" s="19"/>
+      <c r="AH1" s="19"/>
+      <c r="AI1" s="19"/>
+      <c r="AJ1" s="19"/>
+      <c r="AK1" s="19"/>
+      <c r="AL1" s="19"/>
+      <c r="AM1" s="19"/>
+      <c r="AN1" s="19"/>
+      <c r="AO1" s="19"/>
+      <c r="AP1" s="19"/>
     </row>
     <row r="2" spans="1:42" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A2" s="12" t="s">
@@ -742,10 +776,9 @@
       <c r="E2" s="12" t="s">
         <v>5</v>
       </c>
-      <c r="F2" s="15" t="s">
+      <c r="F2" s="13" t="s">
         <v>6</v>
       </c>
-      <c r="G2" s="16"/>
       <c r="H2" s="2"/>
       <c r="I2" s="3"/>
       <c r="J2" s="2"/>
@@ -800,6 +833,14 @@
       <c r="F3" s="6" t="s">
         <v>11</v>
       </c>
+      <c r="M3" s="23" t="s">
+        <v>0</v>
+      </c>
+      <c r="N3" s="24"/>
+      <c r="O3" s="24"/>
+      <c r="P3" s="24"/>
+      <c r="Q3" s="24"/>
+      <c r="R3" s="24"/>
     </row>
     <row r="4" spans="1:42" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A4" s="4"/>
@@ -813,6 +854,24 @@
       <c r="G4" s="4"/>
       <c r="H4" s="7" t="s">
         <v>13</v>
+      </c>
+      <c r="M4" s="12" t="s">
+        <v>1</v>
+      </c>
+      <c r="N4" s="12" t="s">
+        <v>2</v>
+      </c>
+      <c r="O4" s="12" t="s">
+        <v>3</v>
+      </c>
+      <c r="P4" s="12" t="s">
+        <v>4</v>
+      </c>
+      <c r="Q4" s="12" t="s">
+        <v>5</v>
+      </c>
+      <c r="R4" s="13" t="s">
+        <v>6</v>
       </c>
     </row>
     <row r="5" spans="1:42" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
@@ -823,6 +882,24 @@
       <c r="E5" s="4"/>
       <c r="F5" s="4"/>
       <c r="G5" s="4"/>
+      <c r="M5" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="N5" s="4" t="s">
+        <v>8</v>
+      </c>
+      <c r="O5" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="P5" s="4">
+        <v>310</v>
+      </c>
+      <c r="Q5" s="5" t="s">
+        <v>10</v>
+      </c>
+      <c r="R5" s="6" t="s">
+        <v>11</v>
+      </c>
     </row>
     <row r="6" spans="1:42" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A6" s="4" t="s">
@@ -847,6 +924,14 @@
       <c r="H6" s="7" t="s">
         <v>18</v>
       </c>
+      <c r="M6" s="4"/>
+      <c r="N6" s="4" t="s">
+        <v>12</v>
+      </c>
+      <c r="O6" s="4"/>
+      <c r="P6" s="4"/>
+      <c r="Q6" s="4"/>
+      <c r="R6" s="4"/>
     </row>
     <row r="7" spans="1:42" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A7" s="4"/>
@@ -858,6 +943,12 @@
       <c r="E7" s="4"/>
       <c r="F7" s="4"/>
       <c r="G7" s="4"/>
+      <c r="M7" s="4"/>
+      <c r="N7" s="4"/>
+      <c r="O7" s="4"/>
+      <c r="P7" s="4"/>
+      <c r="Q7" s="4"/>
+      <c r="R7" s="4"/>
     </row>
     <row r="8" spans="1:42" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A8" s="4"/>
@@ -869,12 +960,38 @@
       <c r="E8" s="4"/>
       <c r="F8" s="4"/>
       <c r="G8" s="4"/>
-      <c r="H8" s="25" t="s">
+      <c r="H8" s="22" t="s">
         <v>49</v>
+      </c>
+      <c r="M8" s="4" t="s">
+        <v>14</v>
+      </c>
+      <c r="N8" s="4" t="s">
+        <v>15</v>
+      </c>
+      <c r="O8" s="8" t="s">
+        <v>16</v>
+      </c>
+      <c r="P8" s="9">
+        <v>295</v>
+      </c>
+      <c r="Q8" s="10" t="s">
+        <v>17</v>
+      </c>
+      <c r="R8" s="6" t="s">
+        <v>11</v>
       </c>
     </row>
     <row r="9" spans="1:42" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="G9" s="4"/>
+      <c r="M9" s="4"/>
+      <c r="N9" s="4" t="s">
+        <v>19</v>
+      </c>
+      <c r="O9" s="4"/>
+      <c r="P9" s="4"/>
+      <c r="Q9" s="4"/>
+      <c r="R9" s="4"/>
     </row>
     <row r="10" spans="1:42" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A10" s="4" t="s">
@@ -896,9 +1013,17 @@
         <v>11</v>
       </c>
       <c r="G10" s="4"/>
-      <c r="H10" s="25" t="s">
+      <c r="H10" s="22" t="s">
         <v>50</v>
       </c>
+      <c r="M10" s="4"/>
+      <c r="N10" s="4" t="s">
+        <v>20</v>
+      </c>
+      <c r="O10" s="4"/>
+      <c r="P10" s="4"/>
+      <c r="Q10" s="4"/>
+      <c r="R10" s="4"/>
     </row>
     <row r="11" spans="1:42" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A11" s="4"/>
@@ -929,6 +1054,24 @@
         <v>11</v>
       </c>
       <c r="G12" s="4"/>
+      <c r="M12" s="4" t="s">
+        <v>21</v>
+      </c>
+      <c r="N12" s="4" t="s">
+        <v>22</v>
+      </c>
+      <c r="O12" s="4" t="s">
+        <v>23</v>
+      </c>
+      <c r="P12" s="9" t="s">
+        <v>24</v>
+      </c>
+      <c r="Q12" s="10" t="s">
+        <v>17</v>
+      </c>
+      <c r="R12" s="6" t="s">
+        <v>11</v>
+      </c>
     </row>
     <row r="13" spans="1:42" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A13" s="4"/>
@@ -938,6 +1081,12 @@
       <c r="E13" s="4"/>
       <c r="F13" s="4"/>
       <c r="G13" s="4"/>
+      <c r="M13" s="4"/>
+      <c r="N13" s="4"/>
+      <c r="O13" s="4"/>
+      <c r="P13" s="4"/>
+      <c r="Q13" s="4"/>
+      <c r="R13" s="4"/>
     </row>
     <row r="14" spans="1:42" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A14" s="4" t="s">
@@ -959,6 +1108,24 @@
         <v>31</v>
       </c>
       <c r="G14" s="4"/>
+      <c r="M14" s="4" t="s">
+        <v>14</v>
+      </c>
+      <c r="N14" s="4" t="s">
+        <v>25</v>
+      </c>
+      <c r="O14" s="4" t="s">
+        <v>26</v>
+      </c>
+      <c r="P14" s="9">
+        <v>249</v>
+      </c>
+      <c r="Q14" s="10" t="s">
+        <v>17</v>
+      </c>
+      <c r="R14" s="6" t="s">
+        <v>11</v>
+      </c>
     </row>
     <row r="15" spans="1:42" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A15" s="4"/>
@@ -967,6 +1134,12 @@
       <c r="D15" s="4"/>
       <c r="E15" s="4"/>
       <c r="G15" s="4"/>
+      <c r="M15" s="4"/>
+      <c r="N15" s="4"/>
+      <c r="O15" s="4"/>
+      <c r="P15" s="4"/>
+      <c r="Q15" s="4"/>
+      <c r="R15" s="4"/>
     </row>
     <row r="16" spans="1:42" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A16" s="4" t="s">
@@ -988,8 +1161,26 @@
         <v>11</v>
       </c>
       <c r="G16" s="4"/>
-    </row>
-    <row r="17" spans="1:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="M16" s="4" t="s">
+        <v>27</v>
+      </c>
+      <c r="N16" s="4" t="s">
+        <v>28</v>
+      </c>
+      <c r="O16" s="4" t="s">
+        <v>29</v>
+      </c>
+      <c r="P16" s="4">
+        <v>485</v>
+      </c>
+      <c r="Q16" s="11" t="s">
+        <v>30</v>
+      </c>
+      <c r="R16" s="6" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="17" spans="1:18" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A17" s="4"/>
       <c r="B17" s="4"/>
       <c r="C17" s="4"/>
@@ -997,8 +1188,13 @@
       <c r="E17" s="4"/>
       <c r="F17" s="4"/>
       <c r="G17" s="4"/>
-    </row>
-    <row r="18" spans="1:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="M17" s="4"/>
+      <c r="N17" s="4"/>
+      <c r="O17" s="4"/>
+      <c r="P17" s="4"/>
+      <c r="Q17" s="4"/>
+    </row>
+    <row r="18" spans="1:18" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A18" s="4" t="s">
         <v>36</v>
       </c>
@@ -1018,8 +1214,26 @@
         <v>11</v>
       </c>
       <c r="G18" s="4"/>
-    </row>
-    <row r="19" spans="1:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="M18" s="4" t="s">
+        <v>32</v>
+      </c>
+      <c r="N18" s="4" t="s">
+        <v>33</v>
+      </c>
+      <c r="O18" s="4" t="s">
+        <v>34</v>
+      </c>
+      <c r="P18" s="9" t="s">
+        <v>35</v>
+      </c>
+      <c r="Q18" s="11" t="s">
+        <v>30</v>
+      </c>
+      <c r="R18" s="6" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="19" spans="1:18" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A19" s="4"/>
       <c r="B19" s="4"/>
       <c r="C19" s="4"/>
@@ -1027,8 +1241,14 @@
       <c r="E19" s="4"/>
       <c r="F19" s="4"/>
       <c r="G19" s="4"/>
-    </row>
-    <row r="20" spans="1:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="M19" s="4"/>
+      <c r="N19" s="4"/>
+      <c r="O19" s="4"/>
+      <c r="P19" s="4"/>
+      <c r="Q19" s="4"/>
+      <c r="R19" s="4"/>
+    </row>
+    <row r="20" spans="1:18" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A20" s="4" t="s">
         <v>32</v>
       </c>
@@ -1048,8 +1268,26 @@
         <v>41</v>
       </c>
       <c r="G20" s="4"/>
-    </row>
-    <row r="21" spans="1:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="M20" s="4" t="s">
+        <v>36</v>
+      </c>
+      <c r="N20" s="4" t="s">
+        <v>37</v>
+      </c>
+      <c r="O20" s="4" t="s">
+        <v>38</v>
+      </c>
+      <c r="P20" s="9" t="s">
+        <v>39</v>
+      </c>
+      <c r="Q20" s="5" t="s">
+        <v>10</v>
+      </c>
+      <c r="R20" s="6" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="21" spans="1:18" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A21" s="4"/>
       <c r="B21" s="4"/>
       <c r="C21" s="4"/>
@@ -1057,92 +1295,134 @@
       <c r="E21" s="4"/>
       <c r="F21" s="4"/>
       <c r="G21" s="4"/>
-    </row>
-    <row r="22" spans="1:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A22" s="23" t="s">
+      <c r="M21" s="4"/>
+      <c r="N21" s="4"/>
+      <c r="O21" s="4"/>
+      <c r="P21" s="4"/>
+      <c r="Q21" s="4"/>
+      <c r="R21" s="4"/>
+    </row>
+    <row r="22" spans="1:18" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A22" s="20" t="s">
         <v>42</v>
       </c>
-      <c r="B22" s="23" t="s">
+      <c r="B22" s="20" t="s">
         <v>46</v>
       </c>
-      <c r="C22" s="23" t="s">
+      <c r="C22" s="20" t="s">
         <v>43</v>
       </c>
-      <c r="D22" s="23">
+      <c r="D22" s="20">
         <v>500</v>
       </c>
       <c r="E22" s="11" t="s">
         <v>30</v>
       </c>
-      <c r="F22" s="24" t="s">
+      <c r="F22" s="21" t="s">
         <v>44</v>
       </c>
-    </row>
-    <row r="23" spans="1:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A23" s="23"/>
-      <c r="B23" s="23" t="s">
+      <c r="M22" s="4" t="s">
+        <v>32</v>
+      </c>
+      <c r="N22" s="4" t="s">
+        <v>33</v>
+      </c>
+      <c r="O22" s="4" t="s">
+        <v>40</v>
+      </c>
+      <c r="P22" s="9" t="s">
+        <v>35</v>
+      </c>
+      <c r="Q22" s="11" t="s">
+        <v>30</v>
+      </c>
+      <c r="R22" s="6" t="s">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="23" spans="1:18" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A23" s="20"/>
+      <c r="B23" s="20" t="s">
         <v>47</v>
       </c>
-      <c r="C23" s="23"/>
-      <c r="D23" s="23"/>
-      <c r="E23" s="23"/>
-      <c r="F23" s="24" t="s">
+      <c r="C23" s="20"/>
+      <c r="D23" s="20"/>
+      <c r="E23" s="20"/>
+      <c r="F23" s="21" t="s">
         <v>45</v>
       </c>
     </row>
-    <row r="24" spans="1:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A24" s="23"/>
-      <c r="B24" s="23" t="s">
+    <row r="24" spans="1:18" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A24" s="20"/>
+      <c r="B24" s="20" t="s">
         <v>48</v>
       </c>
-      <c r="C24" s="23"/>
-      <c r="D24" s="23"/>
-      <c r="E24" s="23"/>
-      <c r="F24" s="23"/>
-    </row>
-    <row r="25" spans="1:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A25" s="23"/>
-      <c r="B25" s="23"/>
-      <c r="C25" s="23"/>
-      <c r="D25" s="23"/>
-      <c r="E25" s="23"/>
-      <c r="F25" s="23"/>
-    </row>
-    <row r="26" spans="1:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A26" s="23"/>
-      <c r="B26" s="23"/>
-      <c r="C26" s="23"/>
-      <c r="D26" s="23"/>
-      <c r="E26" s="23"/>
-      <c r="F26" s="23"/>
-    </row>
-    <row r="27" spans="1:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A27" s="23"/>
-      <c r="B27" s="23"/>
-      <c r="C27" s="23"/>
-      <c r="D27" s="23"/>
-      <c r="E27" s="23"/>
-      <c r="F27" s="23"/>
-    </row>
-    <row r="28" spans="1:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A28" s="23"/>
-      <c r="B28" s="23"/>
-      <c r="C28" s="23"/>
-      <c r="D28" s="23"/>
-      <c r="E28" s="23"/>
-      <c r="F28" s="23"/>
-    </row>
-    <row r="29" spans="1:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A29" s="23"/>
-      <c r="B29" s="23"/>
-      <c r="C29" s="23"/>
-      <c r="D29" s="23"/>
-      <c r="E29" s="23"/>
-      <c r="F29" s="23"/>
-    </row>
-    <row r="30" spans="1:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="31" spans="1:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="32" spans="1:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+      <c r="C24" s="20"/>
+      <c r="D24" s="20"/>
+      <c r="E24" s="20"/>
+      <c r="F24" s="20"/>
+    </row>
+    <row r="25" spans="1:18" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A25" s="20"/>
+      <c r="B25" s="20"/>
+      <c r="C25" s="20"/>
+      <c r="D25" s="20"/>
+      <c r="E25" s="20"/>
+      <c r="F25" s="20"/>
+    </row>
+    <row r="26" spans="1:18" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A26" s="20" t="s">
+        <v>51</v>
+      </c>
+      <c r="B26" s="20" t="s">
+        <v>53</v>
+      </c>
+      <c r="C26" s="26" t="s">
+        <v>56</v>
+      </c>
+      <c r="D26" s="25" t="s">
+        <v>52</v>
+      </c>
+      <c r="E26" s="10" t="s">
+        <v>17</v>
+      </c>
+      <c r="F26" s="21" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="27" spans="1:18" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A27" s="20"/>
+      <c r="B27" s="20" t="s">
+        <v>54</v>
+      </c>
+      <c r="C27" s="20" t="s">
+        <v>57</v>
+      </c>
+      <c r="D27" s="20"/>
+      <c r="E27" s="20"/>
+      <c r="F27" s="20"/>
+    </row>
+    <row r="28" spans="1:18" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A28" s="20"/>
+      <c r="B28" s="20" t="s">
+        <v>55</v>
+      </c>
+      <c r="C28" s="20"/>
+      <c r="D28" s="20"/>
+      <c r="E28" s="20"/>
+      <c r="F28" s="20"/>
+    </row>
+    <row r="29" spans="1:18" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A29" s="20"/>
+      <c r="B29" s="20"/>
+      <c r="C29" s="20"/>
+      <c r="D29" s="20"/>
+      <c r="E29" s="20"/>
+      <c r="F29" s="20"/>
+    </row>
+    <row r="30" spans="1:18" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="31" spans="1:18" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="32" spans="1:18" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="33" s="1" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="34" s="1" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="35" s="1" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
@@ -2126,31 +2406,41 @@
     <row r="1013" s="1" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="1014" s="1" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
   </sheetData>
-  <mergeCells count="1">
+  <mergeCells count="2">
     <mergeCell ref="A1:F1"/>
+    <mergeCell ref="M3:R3"/>
   </mergeCells>
   <dataValidations count="1">
-    <dataValidation type="list" allowBlank="1" showErrorMessage="1" sqref="E3 E6 E18 E10 E14 E12 E16 E20 E22" xr:uid="{00000000-0002-0000-0000-000000000000}">
+    <dataValidation type="list" allowBlank="1" showErrorMessage="1" sqref="E3 E6 E18 E10 E14 E12 E16 E20 E22 Q5 Q8 Q20 Q12 Q16 Q14 Q18 Q22 E26" xr:uid="{00000000-0002-0000-0000-000000000000}">
       <formula1>"Yes,No,N/A"</formula1>
     </dataValidation>
   </dataValidations>
   <hyperlinks>
-    <hyperlink ref="F3" r:id="rId1" xr:uid="{00000000-0004-0000-0000-000000000000}"/>
-    <hyperlink ref="H4" r:id="rId2" xr:uid="{00000000-0004-0000-0000-000001000000}"/>
-    <hyperlink ref="F6" r:id="rId3" xr:uid="{00000000-0004-0000-0000-000002000000}"/>
-    <hyperlink ref="H6" r:id="rId4" xr:uid="{00000000-0004-0000-0000-000003000000}"/>
-    <hyperlink ref="F10" r:id="rId5" xr:uid="{00000000-0004-0000-0000-000004000000}"/>
-    <hyperlink ref="F12" r:id="rId6" xr:uid="{00000000-0004-0000-0000-000005000000}"/>
-    <hyperlink ref="F14" r:id="rId7" xr:uid="{00000000-0004-0000-0000-000006000000}"/>
-    <hyperlink ref="F16" r:id="rId8" xr:uid="{00000000-0004-0000-0000-000007000000}"/>
-    <hyperlink ref="F18" r:id="rId9" xr:uid="{00000000-0004-0000-0000-000008000000}"/>
-    <hyperlink ref="F20" r:id="rId10" xr:uid="{00000000-0004-0000-0000-000009000000}"/>
-    <hyperlink ref="F22" r:id="rId11" xr:uid="{EA0C5E34-DCD5-474E-8907-E2D257013829}"/>
-    <hyperlink ref="F23" r:id="rId12" xr:uid="{6C8B1E52-79C4-49B7-A348-ED1DC033B22A}"/>
-    <hyperlink ref="H8" r:id="rId13" xr:uid="{9C660D34-92E0-4C03-9408-12824E96A1F4}"/>
-    <hyperlink ref="H10" r:id="rId14" xr:uid="{2B855C48-9DCF-4E59-9FA8-94BCA02C69C0}"/>
+    <hyperlink ref="H4" r:id="rId1" xr:uid="{00000000-0004-0000-0000-000001000000}"/>
+    <hyperlink ref="H6" r:id="rId2" xr:uid="{00000000-0004-0000-0000-000003000000}"/>
+    <hyperlink ref="H8" r:id="rId3" xr:uid="{9C660D34-92E0-4C03-9408-12824E96A1F4}"/>
+    <hyperlink ref="H10" r:id="rId4" xr:uid="{2B855C48-9DCF-4E59-9FA8-94BCA02C69C0}"/>
+    <hyperlink ref="R5" r:id="rId5" xr:uid="{255E628B-5DBF-4212-9B0D-D01F2CCE50B3}"/>
+    <hyperlink ref="R8" r:id="rId6" xr:uid="{F1A81A39-1F77-48D0-8233-C9DAA49408DC}"/>
+    <hyperlink ref="R12" r:id="rId7" xr:uid="{B090B68D-F5C3-43FB-9243-265AB8271C7F}"/>
+    <hyperlink ref="R14" r:id="rId8" xr:uid="{9CCD9474-5B62-4741-9ADE-9689FB2DF395}"/>
+    <hyperlink ref="R16" r:id="rId9" xr:uid="{4E3C373D-34E0-4C23-94DC-9A1E02C8EE43}"/>
+    <hyperlink ref="R18" r:id="rId10" xr:uid="{66A690F7-D389-4FF3-9F85-DF77CD511501}"/>
+    <hyperlink ref="R20" r:id="rId11" xr:uid="{FDBA754D-C7AB-435A-801C-D18FAEB87FEB}"/>
+    <hyperlink ref="R22" r:id="rId12" xr:uid="{A5070469-6AD9-47AC-876E-DAAF29A89B9F}"/>
+    <hyperlink ref="F23" r:id="rId13" xr:uid="{6C8B1E52-79C4-49B7-A348-ED1DC033B22A}"/>
+    <hyperlink ref="F22" r:id="rId14" xr:uid="{EA0C5E34-DCD5-474E-8907-E2D257013829}"/>
+    <hyperlink ref="F20" r:id="rId15" xr:uid="{00000000-0004-0000-0000-000009000000}"/>
+    <hyperlink ref="F18" r:id="rId16" xr:uid="{00000000-0004-0000-0000-000008000000}"/>
+    <hyperlink ref="F16" r:id="rId17" xr:uid="{00000000-0004-0000-0000-000007000000}"/>
+    <hyperlink ref="F14" r:id="rId18" xr:uid="{00000000-0004-0000-0000-000006000000}"/>
+    <hyperlink ref="F12" r:id="rId19" xr:uid="{00000000-0004-0000-0000-000005000000}"/>
+    <hyperlink ref="F10" r:id="rId20" xr:uid="{00000000-0004-0000-0000-000004000000}"/>
+    <hyperlink ref="F6" r:id="rId21" xr:uid="{00000000-0004-0000-0000-000002000000}"/>
+    <hyperlink ref="F3" r:id="rId22" xr:uid="{00000000-0004-0000-0000-000000000000}"/>
+    <hyperlink ref="F26" r:id="rId23" xr:uid="{43E91CE9-9C94-4ADE-A66F-83B2F88CF1DA}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" r:id="rId15"/>
+  <pageSetup orientation="portrait" r:id="rId24"/>
 </worksheet>
 </file>
</xml_diff>